<commit_message>
Add L5 new-lease average block to the Summary tab
Five most recent new-lease contract rents per floor plan by move-in date,
weighted by the 360-unit mix -- the house method from Rent_Chart_Data. Computed
live from the ledger: \$1,892 gross (+0.4% vs the model's \$1,884.7 starting
market rents, which are the prior L5), \$1,866 effective.

Excludes the 12 corporate leases (which would lift it to \$1,933) and the G103
transfer -- the 8/18 roll shows \$2,140 actual against \$1,718 market on that
693sf A1, Ediae's J108->G103 unit transfer, not an arm's-length lease. That
single row is worth +\$31 on the property-wide figure (\$1,923 with it in), so
it is flagged in the workbook for seller confirmation rather than silently
included or dropped.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HqnnqShAVnaRsq64j4w2jf
</commit_message>
<xml_diff>
--- a/SeasonsMeridian/analysis/lease-up/Seasons at Meridian - Lease-Up Analysis.xlsx
+++ b/SeasonsMeridian/analysis/lease-up/Seasons at Meridian - Lease-Up Analysis.xlsx
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1324,7 +1324,7 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>THE CONCESSION STORY</t>
+          <t>L5 NEW LEASE AVERAGE — 5 most recent leases per plan, mix-weighted</t>
         </is>
       </c>
       <c r="B61" s="5" t="n"/>
@@ -1334,95 +1334,270 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>Renewal gross vs effective spread</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="n">
-        <v>0.0888159281170402</v>
+          <t>L5 MIX-WEIGHTED (gross contract rent)</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="n">
+        <v>1892.272222222222</v>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Nearly all renewal economics come from concession burn-off, not rate</t>
+          <t>vs model starting market rent $1,884.7 (the prior L5): +0.4% — starting rents remain current</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>Initial-lease concession FREQUENCY</t>
-        </is>
-      </c>
-      <c r="B63" s="9" t="n">
-        <v>0.75</v>
+          <t xml:space="preserve">  S1_Seas</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="n">
+        <v>1565.2</v>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>255 of 340 initial leases carried a concession (denominator = leases with a computable effective rent)</t>
+          <t>n=5 · newest move-in 2026-08-07 · RRA start $1,496 (+4.6%)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>Initial-lease concession DEPTH</t>
-        </is>
-      </c>
-      <c r="B64" s="9" t="n">
-        <v>0.1000762845941118</v>
+          <t xml:space="preserve">  A1_Seas</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="n">
+        <v>1684</v>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Avg discount among the 255 CONCEDING leases only — $1,963 over 12.7 mo. Spread over all 340 it would read 7.5%</t>
+          <t>n=5 · newest move-in 2026-08-14 · RRA start $1,679 (+0.3%)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>2026 new-lease concession FREQUENCY</t>
-        </is>
-      </c>
-      <c r="B65" s="9" t="n">
-        <v>0.25</v>
+          <t xml:space="preserve">  A2_Seas</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="n">
+        <v>1784.2</v>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>23 of 92 — concessions withdrawn as the asset stabilizes</t>
+          <t>n=5 · newest move-in 2026-08-06 · RRA start $1,766 (+1.0%)</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>2026 new-lease concession DEPTH</t>
-        </is>
-      </c>
-      <c r="B66" s="9" t="n">
-        <v>0.07341246190708824</v>
+          <t xml:space="preserve">  B1_Seas</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="n">
+        <v>1901.8</v>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Avg among the 23 conceding — $1,947 over 14.1 mo</t>
+          <t>n=5 · newest move-in 2026-07-17 · RRA start $1,902 (+0.0%)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">  B2_Seas</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="n">
+        <v>2089</v>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>n=5 · newest move-in 2026-08-16 · RRA start $2,074 (+0.7%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  B3a_Seas</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="n">
+        <v>2068.6</v>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>n=5 · newest move-in 2026-08-16 · RRA start $2,012 (+2.8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  B3b_Seas</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="n">
+        <v>2066.2</v>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>n=5 · newest move-in 2026-07-31 · RRA start $2,066 (+0.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  C1a_Seas</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="n">
+        <v>2477.5</v>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>n=4 · newest move-in 2026-08-03 · RRA start $2,498 (-0.8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  C1b_Seas</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="n">
+        <v>2192.6</v>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>n=5 · newest move-in 2026-07-18 · RRA start $2,266 (-3.3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>Excluded: corporate + one transfer</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>The 12 corporate leases would lift this to $1,933. G103 ($2,140 on a $1,718-market A1) is the Ediae unit TRANSFER, not an arm's-length lease — with it, L5 reads $1,923. Confirm G103's actual charge with the seller.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>THE CONCESSION STORY</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="n"/>
+      <c r="C74" s="5" t="n"/>
+      <c r="D74" s="5" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>Renewal gross vs effective spread</t>
+        </is>
+      </c>
+      <c r="B75" s="10" t="n">
+        <v>0.0888159281170402</v>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Nearly all renewal economics come from concession burn-off, not rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>Initial-lease concession FREQUENCY</t>
+        </is>
+      </c>
+      <c r="B76" s="9" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>255 of 340 initial leases carried a concession (denominator = leases with a computable effective rent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>Initial-lease concession DEPTH</t>
+        </is>
+      </c>
+      <c r="B77" s="9" t="n">
+        <v>0.1000762845941118</v>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Avg discount among the 255 CONCEDING leases only — $1,963 over 12.7 mo. Spread over all 340 it would read 7.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>2026 new-lease concession FREQUENCY</t>
+        </is>
+      </c>
+      <c r="B78" s="9" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>23 of 92 — concessions withdrawn as the asset stabilizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>2026 new-lease concession DEPTH</t>
+        </is>
+      </c>
+      <c r="B79" s="9" t="n">
+        <v>0.07341246190708824</v>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Avg among the 23 conceding — $1,947 over 14.1 mo</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
           <t>2026 renewal concession FREQUENCY</t>
         </is>
       </c>
-      <c r="B67" s="9" t="n">
+      <c r="B80" s="9" t="n">
         <v>0.03125</v>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="D80" s="2" t="inlineStr">
         <is>
           <t>2 of 64 — renewals are written essentially concession-free</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="28" customHeight="1">
-      <c r="A69" s="2" t="inlineStr">
+    <row r="82" ht="28" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>Sources: Yardi rent rolls (1/1, 7/07, 7/19, 8/04, 8/18/2026) · Concession Burn Off (6/21, 7/30/2026) · Renewal Trade-Out report (5/10–7/9/2026) · HelloData Unit Details (8/14/2026) · T12 (Jun 2025–Jul 2026). Measurement date 8/18/2026.</t>
         </is>
@@ -1430,7 +1605,7 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A69:D69"/>
+    <mergeCell ref="A82:D82"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>

</xml_diff>